<commit_message>
modifica funzione creazione archi
</commit_message>
<xml_diff>
--- a/outputs/associations_colored.xlsx
+++ b/outputs/associations_colored.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -493,12 +493,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DU 10-2-484806</t>
+          <t>DU 10-2-562897</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NOVEGRO 1 [DU 1015585. 414 FERROVI]</t>
+          <t>GIUSEPPINA INT AUT B [DU 1035684., BORGOLOMBA]</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
@@ -525,17 +525,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>DU 10-2-512205</t>
+          <t>DU 10-2-320754</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>V. RIVOLTA .</t>
+          <t>SELMO UNO .</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>T01 (250kV A , 2cl)</t>
+          <t>T01 (400kV A , 190cl)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -555,17 +555,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>DU 10-2-408955</t>
+          <t>DU 10-2-274927</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>F. S. DORMITORIO @ B .</t>
+          <t>SELMO 2 .</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>T01 (250kVA, 7cl)</t>
+          <t>T01 (400kV A , 181cl)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -580,58 +580,48 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>UT</t>
+          <t>MB</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AU 10-2-604280</t>
+          <t>DU 10-2-373932</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>AEM DEP FS .</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>U01 (500kW)</t>
-        </is>
-      </c>
+          <t>VIBOLDONE .</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>T01 (160kVA, 15cl)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="I5" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="J5" s="1" t="b">
-        <v>0</v>
+      <c r="H5" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
         <v>4</v>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>MB</t>
-        </is>
-      </c>
+      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
-          <t>DU 10-2-598778</t>
+          <t>DU 10-2-234698</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>V. LAZIO © B .</t>
+          <t>IP AUTOSOLE .</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>T01 (100kVA, 2cl)</t>
+          <t>T01 (100kVA , 2cl)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -646,22 +636,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>MB</t>
+          <t>/\</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>DU 10-2-414140</t>
+          <t>DU 10-2-258590</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>V BASILICATA .</t>
+          <t>VETTABIOLO .</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>T01 (400kV A , 168cl)</t>
+          <t>T01 (25kVA , 12cl)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -676,30 +666,28 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>MB</t>
+          <t>TU</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>DU 10-2-646574</t>
+          <t>DU 10-2-126843</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>V. MICHELANGELO [DU 1050002. A ROLDO]</t>
+          <t>DEP. RANCATE GoW .</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>U01 (507kW)</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="I8" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="J8" s="1" t="b">
-        <v>0</v>
+      <c r="H8" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -713,12 +701,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>DU 00-1-404518</t>
+          <t>DU 00-1-384785</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>PAMBRATE 15</t>
+          <t>MELEG NANO</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
@@ -738,27 +726,23 @@
       <c r="A10" t="n">
         <v>8</v>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>MB</t>
-        </is>
-      </c>
+      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
-          <t>DU 10-2-140439</t>
+          <t>DU 10-2-711076</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>V ABRUZZI 62 TO 1 SOR AF oReh .</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>T02 (250kV A , 198cl)</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
+          <t>BERETTA .</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>U01 (200kW)</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" s="2" t="b">
         <v>1</v>
@@ -775,24 +759,20 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>DU 10-2-465336</t>
+          <t>DU 10-2-416051</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>C SPORTIVO . .</t>
+          <t>IMM. S. GIULIA .</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>T01 (160kV A , 2cl)</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>U01 (220kW)</t>
-        </is>
-      </c>
+          <t>T01 (160kV A , 24cl)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" s="2" t="b">
         <v>1</v>
@@ -809,17 +789,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>DU 10-2-708583</t>
+          <t>DU 10-2-457599</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>REDEST .</t>
+          <t>MUNDUS .</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>T01 (630kV A , 112cl)</t>
+          <t>T01 (100kV A , 6cl)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -839,18 +819,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>DU 10-2-655032</t>
+          <t>DU 10-2-564349</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>DOGANA SCALO .</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
+          <t>SMALTON . ,</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>T01 (160kV A , 13cl)</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>U01 (507kW)</t>
+          <t>U01 (125kW)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
@@ -864,30 +848,28 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>cU</t>
+          <t>MB</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>DU 10-2-206945</t>
+          <t>DU 10-2-192919</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>BUILDING</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
+          <t>PEDRIANO .</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>T01 (100kVA , 47cl)</t>
+        </is>
+      </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="I14" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="J14" s="1" t="b">
-        <v>0</v>
+      <c r="H14" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -896,25 +878,25 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>TU</t>
+          <t>MB</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>DU 10-2-147654</t>
+          <t>DU 10-2-650757</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>MEM STABILIMENTO ate 60kV A , 4cl). .</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>U01 (350kW)</t>
-        </is>
-      </c>
+          <t>MEZZANO .</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>T01 (250kV A , 10cl)</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
       <c r="H15" s="2" t="b">
         <v>1</v>
@@ -926,25 +908,25 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TU</t>
+          <t>MB</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>DU 10-2-371263</t>
+          <t>DU 10-2-256258</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>RAFFAELLO testa ae .</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>U01 (313kW)</t>
-        </is>
-      </c>
+          <t>MONTONE .</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>T01 (100kVA, 10cl)</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
       <c r="H16" s="2" t="b">
         <v>1</v>
@@ -961,17 +943,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>DU 10-2-189364</t>
+          <t>DU 10-2-420767</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>ORSI .</t>
+          <t>RANCATE .</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>T01 (400kV A , 3cl)</t>
+          <t>T01 (160kV A , 18cl)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
@@ -986,25 +968,25 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>cU</t>
+          <t>MB</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>DU 10-2-170799</t>
+          <t>DU 10-2-250549</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>V. CELLINI 3 .</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>U01 (1029kW)</t>
-        </is>
-      </c>
+          <t>COLOG. DUE 6 A .</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>T01 (250kV A , 4cl)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" s="2" t="b">
         <v>1</v>
@@ -1016,25 +998,25 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>TU</t>
+          <t>cU</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>DU 10-2-176761</t>
+          <t>DU 10-2-616671</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>V. MORANDI 56 .</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>T01 (250kV A , 4cl)</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr"/>
+          <t>COLOGNO 2-5 .</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>U01 (500kW)</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" s="2" t="b">
         <v>1</v>
@@ -1051,23 +1033,25 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>DU 10-2-511721</t>
+          <t>DU 10-2-299221</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>V. MORANDI .</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>T01 (200kV A , 5cl)</t>
-        </is>
-      </c>
+          <t>COLOGNO 2-4 [DU 1016005. COLOGNO D</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" s="2" t="b">
-        <v>1</v>
+      <c r="H20" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I20" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J20" s="1" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -1076,28 +1060,30 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>MB</t>
+          <t>cU</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>DU 10-2-396506</t>
+          <t>DU 10-2-495819</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>V . RUGACESIO 8 .</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>T01 (400kVA , 17cl)</t>
-        </is>
-      </c>
+          <t>TIRSO 27 [DU 1016005. COLOGNO DU}</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" s="2" t="b">
-        <v>1</v>
+      <c r="H21" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I21" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J21" s="1" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -1111,16 +1097,24 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>DU 10-2-277462</t>
+          <t>DU 10-2-236151</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Tuite ss Cl). TOD CORY AS, oF 61 (168 KW).</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
+          <t>BESOZZI BIOGAS GOTTOOLW). . .</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>T01 (160kVA , 22cl)</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>U01 (100kW)</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" s="2" t="b">
         <v>1</v>
@@ -1137,305 +1131,23 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>DU 10-2-525086</t>
+          <t>DU 10-2-389187</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>V. TIEPOLO .</t>
+          <t>CASTELLETTO .</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>T01 (400kV A , 20cl)</t>
+          <t>T01 (100kVA , 3cl)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" s="2" t="b">
         <v>1</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>22</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>MB</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>DU 10-2-421460</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>V TIEPOLO .</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>T01 (160kVA, 7cl)</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>23</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>MB</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>DU 10-2-233459</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>CISALPINA [DU 1035408. SEGRATE]</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="I25" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="J25" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>24</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>cU</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>DU 10-2-219834</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>ARAFIN . . .</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>U01 (17kW)</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>G01 (714kV A) \ G02 (714kV A)</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>25</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>TU</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>DU 10-2-223258</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>TUBOPRESS teat ae .</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>U01 (500kW)</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>26</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>cU</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>DU 10-2-366515</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>TURBO 2 .</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>U01 (432kW)</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>27</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>cU</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>DU 10-2-706066</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>RF] .</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>U01 (2500kW)</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>28</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>cU</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>DU 10-2-270426</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>V. RAFFAELLO .</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>U01 (507kW)</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>29</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>TU</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>DU 10-2-491211</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>V . CELLINI .</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>T01 (250kVA, 5cl)</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>30</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>MB</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>UT 0-2-533135</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>5 ,</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>T01 (400kV A , 144cl)</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="I32" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="J32" s="1" t="b">
-        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
aggiunta conversione file pdf
</commit_message>
<xml_diff>
--- a/outputs/associations_colored.xlsx
+++ b/outputs/associations_colored.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -488,17 +488,13 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>MB</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>DU 10-2-562897</t>
-        </is>
-      </c>
+          <t>LUN</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>GIUSEPPINA INT AUT B [DU 1035684., BORGOLOMBA]</t>
+          <t>1-381582</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
@@ -520,28 +516,26 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MB</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>DU 10-2-320754</t>
-        </is>
-      </c>
+          <t>/\</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>SELMO UNO .</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>T01 (400kV A , 190cl)</t>
-        </is>
-      </c>
+          <t>DU 10-2-59675! IN-C. LODOVI T 01 (160kVA , 2'</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" s="2" t="b">
-        <v>1</v>
+      <c r="H3" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I3" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J3" s="1" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -555,17 +549,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>DU 10-2-274927</t>
+          <t>DU 10-2-197005</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>SELMO 2 .</t>
+          <t>IN-BONETTA .</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>T01 (400kV A , 181cl)</t>
+          <t>T01 (250kVA, 145cl)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -585,17 +579,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>DU 10-2-373932</t>
+          <t>DU 10-2-148044</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>VIBOLDONE .</t>
+          <t>IN-V. D. VIOLE .</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>T01 (160kVA, 15cl)</t>
+          <t>T01 (250kV A , 279cl)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -608,20 +602,24 @@
       <c r="A6" t="n">
         <v>4</v>
       </c>
-      <c r="B6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>DU 10-2-234698</t>
+          <t>DU 10-2-606052</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>IP AUTOSOLE .</t>
+          <t>IN-CEREDA .</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>T01 (100kVA , 2cl)</t>
+          <t>T01 (250kVA , 122cl)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -634,24 +632,20 @@
       <c r="A7" t="n">
         <v>5</v>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>/\</t>
-        </is>
-      </c>
+      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
-          <t>DU 10-2-258590</t>
+          <t>DU 10-2-152045</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>VETTABIOLO .</t>
+          <t>IN-PIROGALLA .</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>T01 (25kVA , 12cl)</t>
+          <t>T01 (50kVA, 19cl)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -666,25 +660,25 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>TU</t>
+          <t>MB</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>DU 10-2-126843</t>
+          <t>DU 10-2-134210</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>DEP. RANCATE GoW .</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>U01 (507kW)</t>
-        </is>
-      </c>
+          <t>IN-SIVIR 2 .</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>T01 (250kV A , 173cl)</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" s="2" t="b">
         <v>1</v>
@@ -696,54 +690,64 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>/\</t>
+          <t>MB</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>DU 00-1-384785</t>
+          <t>DU 10-2-169292</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MELEG NANO</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
+          <t>IN-COITAGRO ,</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>T01 (160kVA , 2cl)</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="I9" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="J9" s="1" t="b">
-        <v>0</v>
+      <c r="H9" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
         <v>8</v>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TU</t>
+        </is>
+      </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>DU 10-2-711076</t>
+          <t>DU 10-2-559562</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>BERETTA .</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
+          <t>PO-CONSOR. H 20 . , . . .</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>T01 (250kVA, 14cl)</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>U01 (200kW)</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
+          <t>U01 (761kW)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>G01 (60kVA) \ G02 (100kV A) \ G03 (72kVA )</t>
+        </is>
+      </c>
       <c r="H10" s="2" t="b">
         <v>1</v>
       </c>
@@ -754,22 +758,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>TU</t>
+          <t>MB</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>DU 10-2-416051</t>
+          <t>DU 10-2-414474</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>IMM. S. GIULIA .</t>
+          <t>PO-GENERAL QIL .</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>T01 (160kV A , 24cl)</t>
+          <t>T01 (400kV A , 9cl)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
@@ -784,25 +788,25 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>MB</t>
+          <t>cU</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>DU 10-2-457599</t>
+          <t>DU 10-2-702551</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>MUNDUS .</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>T01 (100kV A , 6cl)</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
+          <t>PO-TRASPORTI VERCESI .</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>U01 (1000kW)</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" s="2" t="b">
         <v>1</v>
@@ -814,29 +818,25 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>TU</t>
+          <t>/\</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>DU 10-2-564349</t>
+          <t>DU 10-2-302167</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>SMALTON . ,</t>
+          <t>IN-METANO .</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>T01 (160kV A , 13cl)</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>U01 (125kW)</t>
-        </is>
-      </c>
+          <t>T01 (50kVA , 3cl)</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" s="2" t="b">
         <v>1</v>
@@ -848,25 +848,25 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>MB</t>
+          <t>TU</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>DU 10-2-192919</t>
+          <t>DU 10-2-303188</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>PEDRIANO .</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>T01 (100kVA , 47cl)</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
+          <t>PQ-STAMP T 01 LOO Ach . .</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>U01 (594kW ) \ U02 (900kW)</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" s="2" t="b">
         <v>1</v>
@@ -878,25 +878,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MB</t>
+          <t>TU</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>DU 10-2-650757</t>
+          <t>DU 10-2-431694</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>MEZZANO .</t>
+          <t>IN-CANEVA . .</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>T01 (250kV A , 10cl)</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
+          <t>T01 (100kVA , 9cl)</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>U01 (225kW)</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" s="2" t="b">
         <v>1</v>
@@ -913,17 +917,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>DU 10-2-256258</t>
+          <t>DU 10-2-390125</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>MONTONE .</t>
+          <t>PO-V, M. TE GRAPPA .</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>T01 (100kVA, 10cl)</t>
+          <t>T01 (250kV A , 162cl)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
@@ -943,17 +947,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>DU 10-2-420767</t>
+          <t>DU 10-2-319452</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>RANCATE .</t>
+          <t>POQO-CROCICCHI .</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>T01 (160kV A , 18cl)</t>
+          <t>T01 (250kKVA , 25cl)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
@@ -973,17 +977,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>DU 10-2-250549</t>
+          <t>DU 10-2-226592</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>COLOG. DUE 6 A .</t>
+          <t>IN-PADANA ,</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>T01 (250kV A , 4cl)</t>
+          <t>T01 (63kKVA, 10cl)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
@@ -998,25 +1002,25 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>cU</t>
+          <t>MB</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>DU 10-2-616671</t>
+          <t>DU 10-2-453962</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>COLOGNO 2-5 .</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>U01 (500kW)</t>
-        </is>
-      </c>
+          <t>PQ-V_ SIENA .</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>T01 (630kV A , 6cl)</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" s="2" t="b">
         <v>1</v>
@@ -1033,25 +1037,23 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>DU 10-2-299221</t>
+          <t>DU 10-2-617074</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>COLOGNO 2-4 [DU 1016005. COLOGNO D</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
+          <t>PQ-V . PUECHER .</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>T01 (400 KVA , 21cl)</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="I20" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="J20" s="1" t="b">
-        <v>0</v>
+      <c r="H20" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -1060,30 +1062,28 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>cU</t>
+          <t>/</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>DU 10-2-495819</t>
+          <t>DU 10-2-262241</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>TIRSO 27 [DU 1016005. COLOGNO DU}</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr"/>
+          <t>IN-MONASTERO .</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>T01 (100kVA , 16cl)</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="I21" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="J21" s="1" t="b">
-        <v>0</v>
+      <c r="H21" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -1097,24 +1097,16 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>DU 10-2-236151</t>
+          <t>DU 10-2-616623</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>BESOZZI BIOGAS GOTTOOLW). . .</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>T01 (160kVA , 22cl)</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>U01 (100kW)</t>
-        </is>
-      </c>
+          <t>PO-GRANATA Gp A 620). UOL{F).</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
       <c r="H22" s="2" t="b">
         <v>1</v>
@@ -1126,27 +1118,1093 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>MB</t>
+          <t>TU</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>DU 10-2-389187</t>
+          <t>DU 10-2-570604</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>CASTELLETTO .</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>T01 (100kVA , 3cl)</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr"/>
+          <t>PQO-MAR. CARNI rate 60kV A, 3cl). .</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>U01 (350kW)</t>
+        </is>
+      </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>DU 10-2-235206</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>IN-WALDIMMOB. .</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>T01 (630kVA , 33cl)</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>DU 10-2-167634</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>IN-CROSINA SUD .</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>T01 (250kV A , 6cl)</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>DU 10-2-376020</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>PO-CE. SPORTIVO .</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>T01 (250kV A , 108cl)</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>DU 10-2-151934</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>PQ-FA RINOTTI .</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>T01 (400kV A , 279cl)</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>TU</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>DU 10-2-195853</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>PQ-PLASTICA Oats DORW yO .</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>U03 (200kW )</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>DU 10-2-418601</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>IN-SCOLAS .</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>T01 (630kVA, 72cl)</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>U 10-2-354425 N-CROSINA NORD 01 (400kVA, 5cl).</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I30" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J30" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>DU 10-2-514382</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>PQ-V, MICCA .</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>T01 (400kV A , 240cl)</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>DU 10-2-309396</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>PO-C FIAMMA .</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>T01 (400kV A , 272cl)</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>DU 10-2-181468</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>IN-VIA LEOPARDI ,</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>T01 (400kVA, 14cl)</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>DU 10-2-748854</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>KATIA .</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>T01 (400kV A , 28cl)</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>DU 10-2-646066</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>PO-LA BAIA .</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>T01 (250kV A , 177cl)</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>DU 10-2-351895</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>PO-NEW GRAF .</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>T01 (250kVA , 172cl)</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>DU 10-2-547667</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>IN-GIESSE .</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>T01 (400kV A , 8cl)</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>36</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>DU 10-2-139614</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>PO-Y BATTISTI .</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>T01 (400kV A , 252cl)</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>DU 10-2-306308</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>PO-V. OBERDAN .</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>T01 (160kV A , 256cl)</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>DU 10-2-664366</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>PQ-PF 048 .</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>T01 (100kVA, 1cl)</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>DU 10-2-147520</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>IN-ARCO .</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>T01 (250kV A , 132cl)</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>DU 10-2-332129</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>PO-V BELLI .</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>T01 (250kV A, 111cl)</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>DU 10-2-476131</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>PQ-V . FOGAZZARO .</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>T01 (250kVA , 101cl)</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>cU</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>DU 10-2-434287</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>IN-BOCCACCIO .</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>U01 (160kW)</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>DU 10-2-168221</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>PO-V . CEREDA .</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>T01 (160kV A , 180cl)</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>DU 10-2-605162</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>IN-C. GIULIA [DU 1035195. INZA GO]</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I46" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J46" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>45</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>TU</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>DU 10-2-598513</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>PO-TOTALERG . . MB ,</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>T01 (160kV A 041)</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>U01 (150kW)</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>G01 (8, 06kV A)</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>46</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>TU</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>DU 10-2-635604</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>PO-FERRERO [DU 1028820. FERRERO]</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I48" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J48" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>47</v>
+      </c>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>DU 10-2-511731</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>PO-V. C. SOLCIA .</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>T01 (50kV A , 6cl)</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>48</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>/\</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>DU 10-2-477916</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>PO-POZ. H 20 .</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>T01 (50kVA , 1cl)</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>49</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>TU</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>DU 10-2-192400</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>PO-PASSONI . . . .</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>T01 (250kVA, 7cl)</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>U01 (59kW)</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>G01 (100kVA) \ G02 (100kVA)</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>50</v>
+      </c>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>DU 10-2-647756</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>BZ-ENERGETICA . .</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>U01 (60kW)</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>G01 (300kV A)</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>51</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>/\</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>DU 10-2-456388</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>PQ-TEM Piola .</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>T01 (100kV A, 2cl)</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>52</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>/\</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>DU 10-2-624742</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>PO-C,. PIOLA .</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>T01 (100kV A , 20cl)</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>DU 10-2-201745</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>BZ-CENTRO INT AUT BT [DU 1034692;GESSATE]</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I55" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J55" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>54</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>/\</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>DU 10-2-161985</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>BZ-C. SOLCIA .</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>T01 (100kVA, 25cl)</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>55</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>/\</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>DU 10-2-518240</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>BZ-V. S. GIORGIO .</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>T01 (160kVA, 172cl)</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>56</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>DU 10-2-450624</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>BZ-C. SPORTIVO .</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>T01 (160kVA, 101cl)</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" s="2" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>